<commit_message>
feat: improve import compatibility and add CEPOD filtering
</commit_message>
<xml_diff>
--- a/public/synthetic-logbook.xlsx
+++ b/public/synthetic-logbook.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="35">
   <si>
     <t>Operation Date</t>
   </si>
@@ -102,6 +102,18 @@
   </si>
   <si>
     <t>Synthetic procedure B</t>
+  </si>
+  <si>
+    <t>Synthetic category A</t>
+  </si>
+  <si>
+    <t>Synthetic category B</t>
+  </si>
+  <si>
+    <t>Synthetic unfamiliar category</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
 </sst>
 </file>
@@ -217,6 +229,9 @@
       <c r="C2" t="s">
         <v>24</v>
       </c>
+      <c r="H2" t="s">
+        <v>31</v>
+      </c>
       <c r="I2" t="s">
         <v>23</v>
       </c>
@@ -231,6 +246,9 @@
       <c r="C3" t="s">
         <v>24</v>
       </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
       <c r="I3" t="s">
         <v>25</v>
       </c>
@@ -245,6 +263,9 @@
       <c r="C4" t="s">
         <v>27</v>
       </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
       <c r="I4" t="s">
         <v>26</v>
       </c>
@@ -259,6 +280,9 @@
       <c r="C5" t="s">
         <v>24</v>
       </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
       <c r="I5" t="s">
         <v>28</v>
       </c>
@@ -273,6 +297,9 @@
       <c r="C6" t="s">
         <v>24</v>
       </c>
+      <c r="H6">
+        <v>7</v>
+      </c>
       <c r="I6" t="s">
         <v>28</v>
       </c>
@@ -295,6 +322,9 @@
       <c r="B8" t="s">
         <v>22</v>
       </c>
+      <c r="H8" t="s">
+        <v>33</v>
+      </c>
       <c r="I8" t="s">
         <v>29</v>
       </c>
@@ -309,6 +339,9 @@
       <c r="C9" t="s">
         <v>27</v>
       </c>
+      <c r="H9" t="s">
+        <v>34</v>
+      </c>
       <c r="I9" t="s">
         <v>23</v>
       </c>
@@ -319,6 +352,9 @@
       </c>
       <c r="C10" t="s">
         <v>24</v>
+      </c>
+      <c r="H10" t="s">
+        <v>31</v>
       </c>
       <c r="I10" t="s">
         <v>23</v>

</xml_diff>